<commit_message>
updated schedule, gitignore, remove Quarto cache
</commit_message>
<xml_diff>
--- a/docs/schedule.xlsx
+++ b/docs/schedule.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jenfra/NBISCourses/scRNAseq/workshop-scRNAseq/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xsinad/Documents/Codes/workshop-scRNAseq/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{989E5B84-3CA6-1B44-9F9B-E5D06AA00DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0ED9A47-F571-A94D-AAAE-6AB22126ACA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19000" yWindow="500" windowWidth="32200" windowHeight="25700" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34560" yWindow="600" windowWidth="32200" windowHeight="25700" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -134,9 +134,6 @@
     <t>Lecture: Batch correction + Integration</t>
   </si>
   <si>
-    <t>lectures/integration.pdf</t>
-  </si>
-  <si>
     <t>Lab: Data integration</t>
   </si>
   <si>
@@ -279,6 +276,9 @@
   </si>
   <si>
     <t>16/04/2026</t>
+  </si>
+  <si>
+    <t>lectures/integration/index.html</t>
   </si>
 </sst>
 </file>
@@ -778,10 +778,10 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C2" s="2">
         <v>0.375</v>
@@ -793,7 +793,7 @@
         <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>14</v>
@@ -808,7 +808,7 @@
         <v>0.4375</v>
       </c>
       <c r="E3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F3" t="s">
         <v>18</v>
@@ -869,7 +869,7 @@
         <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H7" t="s">
         <v>22</v>
@@ -887,7 +887,7 @@
         <v>23</v>
       </c>
       <c r="F8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I8" t="s">
         <v>24</v>
@@ -915,7 +915,7 @@
         <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H10" t="s">
         <v>26</v>
@@ -929,16 +929,16 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="E11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J11" s="3"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C12" s="2">
         <v>0.375</v>
@@ -947,7 +947,7 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J12" s="3"/>
     </row>
@@ -962,7 +962,7 @@
         <v>27</v>
       </c>
       <c r="F13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H13" t="s">
         <v>28</v>
@@ -991,7 +991,7 @@
         <v>29</v>
       </c>
       <c r="F15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I15" t="s">
         <v>24</v>
@@ -1020,10 +1020,10 @@
         <v>30</v>
       </c>
       <c r="F17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H17" t="s">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="K17" s="3"/>
     </row>
@@ -1035,10 +1035,10 @@
         <v>0.625</v>
       </c>
       <c r="E18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I18" t="s">
         <v>24</v>
@@ -1064,13 +1064,13 @@
         <v>0.6875</v>
       </c>
       <c r="E20" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F20" t="s">
         <v>13</v>
       </c>
       <c r="H20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
@@ -1081,16 +1081,16 @@
         <v>0.70833333333333304</v>
       </c>
       <c r="E21" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J21" s="3"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C22" s="2">
         <v>0.375</v>
@@ -1099,7 +1099,7 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J22" s="3"/>
     </row>
@@ -1111,10 +1111,10 @@
         <v>0.4375</v>
       </c>
       <c r="E23" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F23" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I23" t="s">
         <v>24</v>
@@ -1140,16 +1140,16 @@
         <v>0.5</v>
       </c>
       <c r="E25" t="s">
+        <v>35</v>
+      </c>
+      <c r="F25" t="s">
+        <v>53</v>
+      </c>
+      <c r="H25" t="s">
         <v>36</v>
       </c>
-      <c r="F25" t="s">
-        <v>54</v>
-      </c>
-      <c r="H25" t="s">
-        <v>37</v>
-      </c>
       <c r="I25" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K25" s="3"/>
     </row>
@@ -1173,13 +1173,13 @@
         <v>0.58333333333333304</v>
       </c>
       <c r="E27" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F27" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H27" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
@@ -1190,16 +1190,16 @@
         <v>0.60416666666666696</v>
       </c>
       <c r="E28" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F28" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K28" s="3"/>
     </row>
@@ -1222,10 +1222,10 @@
         <v>0.6875</v>
       </c>
       <c r="E30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I30" t="s">
         <v>24</v>
@@ -1239,16 +1239,16 @@
         <v>0.70833333333333304</v>
       </c>
       <c r="E31" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F31" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J31" s="3"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C32" s="2">
         <v>0.375</v>
@@ -1257,7 +1257,7 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E32" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J32" s="3"/>
     </row>
@@ -1269,13 +1269,13 @@
         <v>0.4375</v>
       </c>
       <c r="E33" t="s">
+        <v>39</v>
+      </c>
+      <c r="F33" t="s">
+        <v>54</v>
+      </c>
+      <c r="H33" t="s">
         <v>40</v>
-      </c>
-      <c r="F33" t="s">
-        <v>55</v>
-      </c>
-      <c r="H33" t="s">
-        <v>41</v>
       </c>
       <c r="K33" s="3"/>
     </row>
@@ -1298,10 +1298,10 @@
         <v>0.5</v>
       </c>
       <c r="E35" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F35" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I35" t="s">
         <v>24</v>
@@ -1327,13 +1327,13 @@
         <v>0.58333333333333304</v>
       </c>
       <c r="E37" t="s">
+        <v>42</v>
+      </c>
+      <c r="F37" t="s">
+        <v>65</v>
+      </c>
+      <c r="H37" t="s">
         <v>43</v>
-      </c>
-      <c r="F37" t="s">
-        <v>66</v>
-      </c>
-      <c r="H37" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
@@ -1344,10 +1344,10 @@
         <v>0.63541666666666663</v>
       </c>
       <c r="E38" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F38" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I38" t="s">
         <v>24</v>
@@ -1361,7 +1361,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="E39" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
@@ -1383,13 +1383,13 @@
         <v>0.6875</v>
       </c>
       <c r="E41" t="s">
+        <v>47</v>
+      </c>
+      <c r="F41" t="s">
+        <v>63</v>
+      </c>
+      <c r="H41" t="s">
         <v>48</v>
-      </c>
-      <c r="F41" t="s">
-        <v>64</v>
-      </c>
-      <c r="H41" t="s">
-        <v>49</v>
       </c>
       <c r="J41" s="3"/>
     </row>
@@ -1401,19 +1401,19 @@
         <v>0.70833333333333304</v>
       </c>
       <c r="E42" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F42" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H42" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J42" s="3"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C43" s="2">
         <v>0.375</v>
@@ -1422,13 +1422,13 @@
         <v>0.38541666666666669</v>
       </c>
       <c r="E43" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F43" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H43" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
@@ -1439,10 +1439,10 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="E44" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H44" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
@@ -1453,10 +1453,10 @@
         <v>0.5</v>
       </c>
       <c r="E45" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F45" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
@@ -1479,10 +1479,10 @@
         <v>0.60416666666666663</v>
       </c>
       <c r="E47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F47" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
@@ -1493,10 +1493,10 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="E48" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F48" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="49" spans="3:6" x14ac:dyDescent="0.2">
@@ -1507,10 +1507,10 @@
         <v>0.6875</v>
       </c>
       <c r="E49" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>